<commit_message>
Fix KFall label parsing: F-code offset mapping, merged-cell forward-fill, integer trial IDs
</commit_message>
<xml_diff>
--- a/tests/fixtures/kfall_mock/label_data/SA06_label.xlsx
+++ b/tests/fixtures/kfall_mock/label_data/SA06_label.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>Task Code</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <si>
+    <t>Task Code (Task ID)</t>
   </si>
   <si>
     <t>Description</t>
@@ -31,13 +31,16 @@
     <t>Fall_impact_frame</t>
   </si>
   <si>
-    <t>T22</t>
+    <t>F01 (20)</t>
+  </si>
+  <si>
+    <t>F02 (21)</t>
   </si>
   <si>
     <t>Forward fall when trying to sit down</t>
   </si>
   <si>
-    <t>R01</t>
+    <t>Backward fall when trying to sit down</t>
   </si>
 </sst>
 </file>
@@ -369,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -394,16 +397,110 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
         <v>7</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
       </c>
       <c r="D2">
         <v>140</v>
       </c>
       <c r="E2">
         <v>158</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>150</v>
+      </c>
+      <c r="E3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>145</v>
+      </c>
+      <c r="E4">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>138</v>
+      </c>
+      <c r="E5">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>142</v>
+      </c>
+      <c r="E6">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>122</v>
+      </c>
+      <c r="E7">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>128</v>
+      </c>
+      <c r="E8">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="C9">
+        <v>4</v>
+      </c>
+      <c r="D9">
+        <v>130</v>
+      </c>
+      <c r="E9">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10">
+        <v>133</v>
+      </c>
+      <c r="E10">
+        <v>170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>